<commit_message>
n8n board refresh 2026-07-10T17:38:51Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-19 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-10 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.722</v>
+        <v>0.796</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>66.36</v>
+        <v>62.575</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>0.833</v>
+        <v>0.944</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.044509997</v>
+        <v>0.04565000057220459</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>119934040.26522</v>
+        <v>119934038.3220136</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>66.36</v>
+        <v>62.575</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>7958822912</v>
+        <v>7504872448</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>9.619999999999999</v>
+        <v>9.07</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>9.74</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>1.09</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="6">
@@ -1532,16 +1532,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>14023314432</v>
+        <v>15235529728</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>39.798508</v>
+        <v>43.238804</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>14.457</v>
+        <v>15.114</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.046</v>
+        <v>1.093</v>
       </c>
     </row>
     <row r="7">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>9256183808</v>
+        <v>8608842752</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>16.238672</v>
+        <v>15.411559</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>1.887</v>
+        <v>1.854</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>1.011</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>9628703744</v>
+        <v>10113275904</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>23.303007</v>
+        <v>22.432602</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>12.721</v>
+        <v>13.867</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>2.128</v>
+        <v>2.245</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>15251364864</v>
+        <v>16003362816</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>39.10569</v>
+        <v>41.08955</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>15.852</v>
+        <v>16.38</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>2.958</v>
+        <v>3.057</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>12409547776</v>
+        <v>12718198784</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>39.28702</v>
+        <v>40.264168</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>23.363</v>
+        <v>24.416</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>5.245</v>
+        <v>5.481</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>15191297024</v>
+        <v>12735360000</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>18.006554</v>
+        <v>15.11811</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>13.297</v>
+        <v>10.939</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>3.182</v>
+        <v>2.617</v>
       </c>
     </row>
     <row r="12">
@@ -1676,14 +1676,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>10318899200</v>
+        <v>11621041152</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>7.925</v>
+        <v>8.396000000000001</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>1.639</v>
+        <v>1.737</v>
       </c>
     </row>
     <row r="13">
@@ -1698,16 +1698,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>15131908096</v>
+        <v>14029338624</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>22.01818</v>
+        <v>20.828623</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>86.696</v>
+        <v>81.25</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>57.189</v>
+        <v>53.597</v>
       </c>
     </row>
     <row r="15">
@@ -1761,7 +1761,7 @@
         <v>0.167</v>
       </c>
       <c r="F17" s="35" t="n">
-        <v>0.333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-11T17:39:20Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-10 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-11 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>62.575</v>
+        <v>62.76</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04565000057220459</v>
+        <v>0.04568999767303467</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>119934038.3220136</v>
+        <v>119934033.9069471</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>62.575</v>
+        <v>62.76</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>7504872448</v>
+        <v>7527059968</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>9.07</v>
+        <v>9.1</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>8.710000000000001</v>
+        <v>8.67</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="6">
@@ -1532,10 +1532,10 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>15235529728</v>
+        <v>15219752960</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>43.238804</v>
+        <v>43.19403</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>15.114</v>
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>8608842752</v>
+        <v>8562743296</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>15.411559</v>
+        <v>15.312566</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>1.854</v>
+        <v>1.857</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.994</v>
+        <v>0.995</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>10113275904</v>
+        <v>9971829760</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>22.432602</v>
+        <v>22.118856</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>13.867</v>
+        <v>13.806</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>2.245</v>
+        <v>2.235</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>16003362816</v>
+        <v>16072064000</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>41.08955</v>
+        <v>41.154263</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>16.38</v>
+        <v>16.484</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>3.057</v>
+        <v>3.076</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>12718198784</v>
+        <v>12650348544</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>40.264168</v>
+        <v>40.196335</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>24.416</v>
+        <v>24.63</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>5.481</v>
+        <v>5.529</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>12735360000</v>
+        <v>12600488960</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>15.11811</v>
+        <v>14.958006</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>10.939</v>
+        <v>10.755</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>2.617</v>
+        <v>2.573</v>
       </c>
     </row>
     <row r="12">
@@ -1676,14 +1676,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>11621041152</v>
+        <v>11543735296</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>8.396000000000001</v>
+        <v>8.518000000000001</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>1.737</v>
+        <v>1.762</v>
       </c>
     </row>
     <row r="13">
@@ -1698,16 +1698,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>14029338624</v>
+        <v>14021008384</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>20.828623</v>
+        <v>20.83466</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>81.25</v>
+        <v>81.645</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>53.597</v>
+        <v>53.858</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-13T17:39:30Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-12 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-13 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>62.76</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04568999767303467</v>
+        <v>0.04609000205993653</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>119934033.9069471</v>
+        <v>119934041.2242348</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>62.76</v>
+        <v>64.04000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1508,10 +1508,10 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>7527059968</v>
+        <v>7680576000</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>9.1</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E5" s="31" t="n">
         <v>8.67</v>
@@ -1532,10 +1532,10 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>15219752960</v>
+        <v>15299953664</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>43.19403</v>
+        <v>43.421642</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>15.114</v>
@@ -1556,10 +1556,10 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>8562743296</v>
+        <v>8406276096</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>15.312566</v>
+        <v>15.03276</v>
       </c>
       <c r="E7" s="33" t="n">
         <v>1.857</v>
@@ -1580,10 +1580,10 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>9971829760</v>
+        <v>9727407104</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>22.118856</v>
+        <v>21.576693</v>
       </c>
       <c r="E8" s="33" t="n">
         <v>13.806</v>
@@ -1604,10 +1604,10 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>16072064000</v>
+        <v>16094787584</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>41.154263</v>
+        <v>41.21245</v>
       </c>
       <c r="E9" s="33" t="n">
         <v>16.484</v>
@@ -1628,10 +1628,10 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>12650348544</v>
+        <v>12473553920</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>40.196335</v>
+        <v>39.63457</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>24.63</v>
@@ -1652,10 +1652,10 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>12600488960</v>
+        <v>12432452608</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>14.958006</v>
+        <v>14.758531</v>
       </c>
       <c r="E11" s="33" t="n">
         <v>10.755</v>
@@ -1676,7 +1676,7 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>11543735296</v>
+        <v>11319866368</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
@@ -1698,10 +1698,10 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>14021008384</v>
+        <v>13894567936</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>20.83466</v>
+        <v>20.646772</v>
       </c>
       <c r="E13" s="33" t="n">
         <v>81.645</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-14T17:39:08Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-13 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-14 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.796</v>
+        <v>0.759</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>64.04000000000001</v>
+        <v>64.285</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>0.944</v>
+        <v>0.889</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04609000205993653</v>
+        <v>0.04586999893188477</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>119934041.2242348</v>
+        <v>119934046.6982967</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>64.04000000000001</v>
+        <v>64.285</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>7680576000</v>
+        <v>7709960192</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>9.279999999999999</v>
+        <v>9.32</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>8.67</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="6">
@@ -1532,16 +1532,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>15299953664</v>
+        <v>15185568768</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>43.421642</v>
+        <v>42.77778</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>15.114</v>
+        <v>15.165</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.093</v>
+        <v>1.097</v>
       </c>
     </row>
     <row r="7">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>8406276096</v>
+        <v>8371288576</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>15.03276</v>
+        <v>15.315659</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>1.857</v>
+        <v>1.847</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.995</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>9727407104</v>
+        <v>9748212736</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>21.576693</v>
+        <v>22.137323</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>13.806</v>
+        <v>13.497</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>2.235</v>
+        <v>2.185</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>16094787584</v>
+        <v>15972448256</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>41.21245</v>
+        <v>40.954605</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>16.484</v>
+        <v>16.461</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>3.076</v>
+        <v>3.072</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>12473553920</v>
+        <v>12522729472</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>39.63457</v>
+        <v>39.71795</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>24.63</v>
+        <v>24.291</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>5.529</v>
+        <v>5.453</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>12432452608</v>
+        <v>12828222464</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>14.758531</v>
+        <v>15.188482</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>10.755</v>
+        <v>10.639</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>2.573</v>
+        <v>2.546</v>
       </c>
     </row>
     <row r="12">
@@ -1676,14 +1676,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>11319866368</v>
+        <v>11442269184</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>8.518000000000001</v>
+        <v>8.429</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>1.762</v>
+        <v>1.744</v>
       </c>
     </row>
     <row r="13">
@@ -1698,16 +1698,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>13894567936</v>
+        <v>13300144128</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>20.646772</v>
+        <v>19.763483</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>81.645</v>
+        <v>80.675</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>53.858</v>
+        <v>53.218</v>
       </c>
     </row>
     <row r="15">
@@ -1761,7 +1761,7 @@
         <v>0.167</v>
       </c>
       <c r="F17" s="35" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-23T17:40:13Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-14 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-23 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>64.285</v>
+        <v>65.495</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04586999893188477</v>
+        <v>0.04699000358581543</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>119934046.6982967</v>
+        <v>119934047.6066875</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>64.285</v>
+        <v>65.495</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>7709960192</v>
+        <v>7855080448</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>9.32</v>
+        <v>9.49</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>8.869999999999999</v>
+        <v>8.99</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>0.99</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="6">
@@ -1532,16 +1532,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>15185568768</v>
+        <v>14967316480</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>42.77778</v>
+        <v>42.477608</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>15.165</v>
+        <v>14.88</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.097</v>
+        <v>1.076</v>
       </c>
     </row>
     <row r="7">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>8371288576</v>
+        <v>8141393408</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>15.315659</v>
+        <v>14.465848</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>1.847</v>
+        <v>1.839</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.99</v>
+        <v>0.986</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>9748212736</v>
+        <v>9793115136</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>22.137323</v>
+        <v>21.736877</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>13.497</v>
+        <v>13.743</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>2.185</v>
+        <v>2.225</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>15972448256</v>
+        <v>16152918016</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>40.954605</v>
+        <v>41.417343</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>16.461</v>
+        <v>16.584</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>3.072</v>
+        <v>3.095</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>12522729472</v>
+        <v>12573978624</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>39.71795</v>
+        <v>39.95367</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>24.291</v>
+        <v>24.712</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>5.453</v>
+        <v>5.548</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>12828222464</v>
+        <v>13992313856</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>15.188482</v>
+        <v>17.433884</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>10.639</v>
+        <v>11.267</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>2.546</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="12">
@@ -1676,14 +1676,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>11442269184</v>
+        <v>11027548160</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>8.429</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>1.744</v>
+        <v>1.733</v>
       </c>
     </row>
     <row r="13">
@@ -1698,16 +1698,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>13300144128</v>
+        <v>12946406400</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>19.763483</v>
+        <v>20.545797</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>80.675</v>
+        <v>85.527</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>53.218</v>
+        <v>57.86</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-26T17:39:18Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-25 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-26 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>141.43</v>
+        <v>179.31</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.95</v>
+        <v>1.472</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="8">
@@ -1526,7 +1526,7 @@
         <v>11.39</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.609999999999999</v>
+        <v>9.84</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>1.11</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-27T17:39:07Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-26 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-27 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>179.31</v>
+        <v>180.63</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>72.53</v>
+        <v>73.04000000000001</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.472</v>
+        <v>1.473</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04678999900817871</v>
+        <v>0.04647000312805176</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>119934034.027299</v>
+        <v>119934037.2398686</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>72.53</v>
+        <v>73.04000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>8698815488</v>
+        <v>8759982080</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.39</v>
+        <v>11.47</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>9.84</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>15035684864</v>
+        <v>15175050240</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>42.671642</v>
+        <v>43.06716</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>14.983</v>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>8041387008</v>
+        <v>8170524160</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>14.288155</v>
+        <v>14.51761</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>1.923</v>
@@ -1592,10 +1592,10 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>9882921984</v>
+        <v>9946235904</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>21.936213</v>
+        <v>22.076744</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>13.687</v>
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16051452928</v>
+        <v>15977468928</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>41.15718</v>
+        <v>40.96748</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>16.466</v>
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>13058610176</v>
+        <v>12964484096</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>41.49358</v>
+        <v>41.194496</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>25.374</v>
@@ -1664,10 +1664,10 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14135702528</v>
+        <v>14114690048</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>17.557692</v>
+        <v>17.531593</v>
       </c>
       <c r="E11" s="34" t="n">
         <v>11.723</v>
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>11462401024</v>
+        <v>11496625152</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
@@ -1710,10 +1710,10 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>12869053440</v>
+        <v>12928852992</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.403772</v>
+        <v>20.498585</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>85.044</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-31T17:43:27Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -20,11 +20,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="169" formatCode="+0.0%;-0.0%"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -126,22 +126,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,9 +149,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -596,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -621,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-27 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-31 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.833</v>
+        <v>0.759</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -657,7 +656,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -672,8 +671,10 @@
           <t>DCF intrinsic value / share</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>180.63</v>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>73.04000000000001</v>
+        <v>69.25</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -702,8 +703,10 @@
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>1.473</v>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -726,7 +729,7 @@
           <t>value_score</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="8" t="n">
         <v>0.5</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
@@ -737,8 +740,8 @@
           <t>comps_percentile</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
-        <v>0.833</v>
+      <c r="B14" s="8" t="n">
+        <v>0.889</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -746,67 +749,52 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>dcf_margin</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Normalized (intrinsic − market) / market, clipped ±50%</t>
-        </is>
-      </c>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Honest caveats (read before acting)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Honest caveats (read before acting)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
+          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
+          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
+          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
+          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>This is a SIGNAL screen, not an investment thesis. Verify with primary filings before acting.</t>
         </is>
@@ -816,7 +804,6 @@
   <mergeCells count="11">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
@@ -825,6 +812,7 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -890,8 +878,8 @@
           <t>Risk-free rate (10y Treasury)</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
-        <v>0.04647000312805176</v>
+      <c r="B5" s="9" t="n">
+        <v>0.04736999988555908</v>
       </c>
     </row>
     <row r="6">
@@ -900,7 +888,7 @@
           <t>Equity risk premium (ERP)</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -910,7 +898,7 @@
           <t>Beta (levered)</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -920,7 +908,7 @@
           <t>Credit spread over risk-free</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="9" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -930,7 +918,7 @@
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="9" t="n">
         <v>0.21</v>
       </c>
     </row>
@@ -940,7 +928,7 @@
           <t>Equity weight (cap structure)</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="11" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -950,7 +938,7 @@
           <t>FCF growth (flat, faded avg)</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="9" t="n">
         <v>0.0725</v>
       </c>
     </row>
@@ -960,7 +948,7 @@
           <t>Terminal growth rate</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="9" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -970,7 +958,7 @@
           <t>Latest FCF ($, base year)</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="12" t="n">
         <v>951000000</v>
       </c>
     </row>
@@ -980,7 +968,7 @@
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="13">
         <f>B5+B7*B6</f>
         <v/>
       </c>
@@ -991,18 +979,18 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="13">
         <f>(B5+B8)*(1-B9)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <f>B10*B15+(1-B10)*B16</f>
         <v/>
       </c>
@@ -1049,23 +1037,23 @@
           <t>Projected FCF</t>
         </is>
       </c>
-      <c r="B22" s="17">
+      <c r="B22" s="16">
         <f>$B$13*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="16">
         <f>B22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="16">
         <f>C22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="16">
         <f>D22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="F22" s="17">
+      <c r="F22" s="16">
         <f>E22*(1+$B$11)</f>
         <v/>
       </c>
@@ -1076,23 +1064,23 @@
           <t>Discount factor</t>
         </is>
       </c>
-      <c r="B23" s="18">
+      <c r="B23" s="17">
         <f>1/(1+$B$17)^1</f>
         <v/>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="17">
         <f>1/(1+$B$17)^2</f>
         <v/>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="17">
         <f>1/(1+$B$17)^3</f>
         <v/>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="17">
         <f>1/(1+$B$17)^4</f>
         <v/>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="17">
         <f>1/(1+$B$17)^5</f>
         <v/>
       </c>
@@ -1103,23 +1091,23 @@
           <t>PV of FCF</t>
         </is>
       </c>
-      <c r="B24" s="17">
+      <c r="B24" s="16">
         <f>B22*B23</f>
         <v/>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="16">
         <f>C22*C23</f>
         <v/>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="16">
         <f>D22*D23</f>
         <v/>
       </c>
-      <c r="E24" s="17">
+      <c r="E24" s="16">
         <f>E22*E23</f>
         <v/>
       </c>
-      <c r="F24" s="17">
+      <c r="F24" s="16">
         <f>F22*F23</f>
         <v/>
       </c>
@@ -1130,7 +1118,7 @@
           <t>Sum of PV (explicit 5y)</t>
         </is>
       </c>
-      <c r="B26" s="17">
+      <c r="B26" s="16">
         <f>SUM(B24:F24)</f>
         <v/>
       </c>
@@ -1141,7 +1129,7 @@
           <t>Terminal value (Gordon)</t>
         </is>
       </c>
-      <c r="B27" s="17">
+      <c r="B27" s="16">
         <f>F22*(1+B12)/(B17-B12)</f>
         <v/>
       </c>
@@ -1152,18 +1140,18 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="B28" s="17">
+      <c r="B28" s="16">
         <f>B27/(1+B17)^5</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B29" s="20">
+      <c r="B29" s="19">
         <f>B26+B28</f>
         <v/>
       </c>
@@ -1188,7 +1176,7 @@
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n">
+      <c r="B32" s="12" t="n">
         <v>4160000000</v>
       </c>
     </row>
@@ -1198,7 +1186,7 @@
           <t>Plus: cash &amp; ST investments</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="12" t="n">
         <v>540000000</v>
       </c>
     </row>
@@ -1208,7 +1196,7 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="B34" s="17">
+      <c r="B34" s="16">
         <f>B29-B32+B33</f>
         <v/>
       </c>
@@ -1219,17 +1207,17 @@
           <t>Diluted shares outstanding</t>
         </is>
       </c>
-      <c r="B35" s="21" t="n">
-        <v>119934037.2398686</v>
+      <c r="B35" s="20" t="n">
+        <v>120284976.9819495</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Intrinsic per share</t>
         </is>
       </c>
-      <c r="B36" s="22">
+      <c r="B36" s="21">
         <f>B34/B35</f>
         <v/>
       </c>
@@ -1240,17 +1228,17 @@
           <t>Current market price</t>
         </is>
       </c>
-      <c r="B37" s="23" t="n">
-        <v>73.04000000000001</v>
+      <c r="B37" s="22" t="n">
+        <v>69.25</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B38" s="24">
+      <c r="B38" s="23">
         <f>(B36-B37)/B37</f>
         <v/>
       </c>
@@ -1270,158 +1258,158 @@
       <c r="H41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="inlineStr">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>WACC ↓ / TermG →</t>
         </is>
       </c>
-      <c r="B42" s="26">
+      <c r="B42" s="25">
         <f>$B$12+-0.01</f>
         <v/>
       </c>
-      <c r="C42" s="26">
+      <c r="C42" s="25">
         <f>$B$12+-0.005</f>
         <v/>
       </c>
-      <c r="D42" s="26">
+      <c r="D42" s="25">
         <f>$B$12+0.0</f>
         <v/>
       </c>
-      <c r="E42" s="26">
+      <c r="E42" s="25">
         <f>$B$12+0.005</f>
         <v/>
       </c>
-      <c r="F42" s="26">
+      <c r="F42" s="25">
         <f>$B$12+0.01</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="26">
+      <c r="A43" s="25">
         <f>$B$17+-0.01</f>
         <v/>
       </c>
-      <c r="B43" s="27">
+      <c r="B43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A43-B$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C43" s="27">
+      <c r="C43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A43-C$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D43" s="27">
+      <c r="D43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A43-D$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E43" s="27">
+      <c r="E43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A43-E$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F43" s="27">
+      <c r="F43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A43-F$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="26">
+      <c r="A44" s="25">
         <f>$B$17+-0.005</f>
         <v/>
       </c>
-      <c r="B44" s="27">
+      <c r="B44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A44-B$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C44" s="27">
+      <c r="C44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A44-C$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D44" s="27">
+      <c r="D44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A44-D$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E44" s="27">
+      <c r="E44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A44-E$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F44" s="27">
+      <c r="F44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A44-F$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="26">
+      <c r="A45" s="25">
         <f>$B$17+0.0</f>
         <v/>
       </c>
-      <c r="B45" s="27">
+      <c r="B45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A45-B$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C45" s="27">
+      <c r="C45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A45-C$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D45" s="28">
+      <c r="D45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A45-D$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E45" s="27">
+      <c r="E45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A45-E$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F45" s="27">
+      <c r="F45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A45-F$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="26">
+      <c r="A46" s="25">
         <f>$B$17+0.005</f>
         <v/>
       </c>
-      <c r="B46" s="27">
+      <c r="B46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A46-B$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C46" s="27">
+      <c r="C46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A46-C$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D46" s="27">
+      <c r="D46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A46-D$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E46" s="27">
+      <c r="E46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A46-E$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F46" s="27">
+      <c r="F46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A46-F$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="26">
+      <c r="A47" s="25">
         <f>$B$17+0.01</f>
         <v/>
       </c>
-      <c r="B47" s="27">
+      <c r="B47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A47-B$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C47" s="27">
+      <c r="C47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A47-C$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D47" s="27">
+      <c r="D47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A47-D$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E47" s="27">
+      <c r="E47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A47-E$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F47" s="27">
+      <c r="F47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A47-F$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
@@ -1477,59 +1465,59 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>P/E (TTM)</t>
         </is>
       </c>
-      <c r="E4" s="29" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="F4" s="29" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>EV/Revenue</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>BAH</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Booz Allen Hamilton Holding Corporation</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="n">
-        <v>8759982080</v>
-      </c>
-      <c r="D5" s="32" t="n">
-        <v>11.47</v>
-      </c>
-      <c r="E5" s="32" t="n">
-        <v>9.84</v>
-      </c>
-      <c r="F5" s="32" t="n">
-        <v>1.11</v>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Booz Allen Hamilton Holding Cor</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="n">
+        <v>8329734656</v>
+      </c>
+      <c r="D5" s="31" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="E5" s="31" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="F5" s="31" t="n">
+        <v>1.07</v>
       </c>
     </row>
     <row r="6">
@@ -1543,17 +1531,17 @@
           <t>Aramark</t>
         </is>
       </c>
-      <c r="C6" s="33" t="n">
-        <v>15175050240</v>
-      </c>
-      <c r="D6" s="34" t="n">
-        <v>43.06716</v>
-      </c>
-      <c r="E6" s="34" t="n">
-        <v>14.983</v>
-      </c>
-      <c r="F6" s="34" t="n">
-        <v>1.084</v>
+      <c r="C6" s="32" t="n">
+        <v>15031741440</v>
+      </c>
+      <c r="D6" s="33" t="n">
+        <v>42.660446</v>
+      </c>
+      <c r="E6" s="33" t="n">
+        <v>14.996</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <v>1.085</v>
       </c>
     </row>
     <row r="7">
@@ -1567,17 +1555,15 @@
           <t>Grupo Aeroportuario del Sureste</t>
         </is>
       </c>
-      <c r="C7" s="33" t="n">
-        <v>8170524160</v>
-      </c>
-      <c r="D7" s="34" t="n">
-        <v>14.51761</v>
-      </c>
-      <c r="E7" s="34" t="n">
-        <v>1.923</v>
-      </c>
-      <c r="F7" s="34" t="n">
-        <v>0.993</v>
+      <c r="C7" s="32" t="n"/>
+      <c r="D7" s="33" t="n">
+        <v>14.910694</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>1.937</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1591,17 +1577,17 @@
           <t>Acuity Inc.</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
-        <v>9946235904</v>
-      </c>
-      <c r="D8" s="34" t="n">
-        <v>22.076744</v>
-      </c>
-      <c r="E8" s="34" t="n">
-        <v>13.687</v>
-      </c>
-      <c r="F8" s="34" t="n">
-        <v>2.216</v>
+      <c r="C8" s="32" t="n">
+        <v>9940698112</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <v>22.03517</v>
+      </c>
+      <c r="E8" s="33" t="n">
+        <v>13.995</v>
+      </c>
+      <c r="F8" s="33" t="n">
+        <v>2.266</v>
       </c>
     </row>
     <row r="9">
@@ -1615,17 +1601,17 @@
           <t>Clean Harbors, Inc.</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
-        <v>15977468928</v>
-      </c>
-      <c r="D9" s="34" t="n">
-        <v>40.96748</v>
-      </c>
-      <c r="E9" s="34" t="n">
-        <v>16.466</v>
-      </c>
-      <c r="F9" s="34" t="n">
-        <v>3.073</v>
+      <c r="C9" s="32" t="n">
+        <v>16626399232</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>38.17818</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>16.126</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <v>3.086</v>
       </c>
     </row>
     <row r="10">
@@ -1639,17 +1625,15 @@
           <t>Crane Company</t>
         </is>
       </c>
-      <c r="C10" s="33" t="n">
-        <v>12964484096</v>
-      </c>
-      <c r="D10" s="34" t="n">
-        <v>41.194496</v>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>25.374</v>
-      </c>
-      <c r="F10" s="34" t="n">
-        <v>5.696</v>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="33" t="n">
+        <v>37.66899</v>
+      </c>
+      <c r="E10" s="33" t="n">
+        <v>24.719</v>
+      </c>
+      <c r="F10" s="33" t="n">
+        <v>5.058</v>
       </c>
     </row>
     <row r="11">
@@ -1663,17 +1647,17 @@
           <t>Mueller Industries, Inc.</t>
         </is>
       </c>
-      <c r="C11" s="33" t="n">
-        <v>14114690048</v>
-      </c>
-      <c r="D11" s="34" t="n">
-        <v>17.531593</v>
-      </c>
-      <c r="E11" s="34" t="n">
-        <v>11.723</v>
-      </c>
-      <c r="F11" s="34" t="n">
-        <v>2.74</v>
+      <c r="C11" s="32" t="n">
+        <v>14857861120</v>
+      </c>
+      <c r="D11" s="33" t="n">
+        <v>17.49349</v>
+      </c>
+      <c r="E11" s="33" t="n">
+        <v>12.322</v>
+      </c>
+      <c r="F11" s="33" t="n">
+        <v>2.88</v>
       </c>
     </row>
     <row r="12">
@@ -1687,15 +1671,15 @@
           <t>Owens Corning Inc</t>
         </is>
       </c>
-      <c r="C12" s="33" t="n">
-        <v>11496625152</v>
-      </c>
-      <c r="D12" s="34" t="n"/>
-      <c r="E12" s="34" t="n">
-        <v>8.478</v>
-      </c>
-      <c r="F12" s="34" t="n">
-        <v>1.754</v>
+      <c r="C12" s="32" t="n">
+        <v>11164849152</v>
+      </c>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="33" t="n">
+        <v>8.339</v>
+      </c>
+      <c r="F12" s="33" t="n">
+        <v>1.725</v>
       </c>
     </row>
     <row r="13">
@@ -1709,17 +1693,17 @@
           <t>Grupo Aeroportuario Del Pacific</t>
         </is>
       </c>
-      <c r="C13" s="33" t="n">
-        <v>12928852992</v>
-      </c>
-      <c r="D13" s="34" t="n">
-        <v>20.498585</v>
-      </c>
-      <c r="E13" s="34" t="n">
-        <v>85.044</v>
-      </c>
-      <c r="F13" s="34" t="n">
-        <v>57.533</v>
+      <c r="C13" s="32" t="n">
+        <v>12923200512</v>
+      </c>
+      <c r="D13" s="33" t="n">
+        <v>20.528357</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>86.309</v>
+      </c>
+      <c r="F13" s="33" t="n">
+        <v>58.389</v>
       </c>
     </row>
     <row r="15">
@@ -1728,15 +1712,15 @@
           <t>Peer median</t>
         </is>
       </c>
-      <c r="D15" s="35">
+      <c r="D15" s="34">
         <f>MEDIAN(D6:D13)</f>
         <v/>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="34">
         <f>MEDIAN(E6:E13)</f>
         <v/>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="34">
         <f>MEDIAN(F6:F13)</f>
         <v/>
       </c>
@@ -1747,15 +1731,15 @@
           <t>Peer mean</t>
         </is>
       </c>
-      <c r="D16" s="35">
+      <c r="D16" s="34">
         <f>AVERAGE(D6:D13)</f>
         <v/>
       </c>
-      <c r="E16" s="35">
+      <c r="E16" s="34">
         <f>AVERAGE(E6:E13)</f>
         <v/>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="34">
         <f>AVERAGE(F6:F13)</f>
         <v/>
       </c>
@@ -1766,14 +1750,14 @@
           <t>Target percentile vs peers</t>
         </is>
       </c>
-      <c r="D17" s="36" t="n">
+      <c r="D17" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="36" t="n">
+      <c r="E17" s="35" t="n">
         <v>0.167</v>
       </c>
-      <c r="F17" s="36" t="n">
-        <v>0.333</v>
+      <c r="F17" s="35" t="n">
+        <v>0.167</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-03T17:42:05Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -20,11 +20,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.0000"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -126,21 +126,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,9 +150,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -595,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -620,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-31 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-03 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.759</v>
+        <v>0.833</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -656,7 +657,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -671,10 +672,8 @@
           <t>DCF intrinsic value / share</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B8" s="7" t="n">
+        <v>178.33</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -689,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>69.25</v>
+        <v>71.36</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,10 +702,8 @@
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B10" s="8" t="n">
+        <v>1.499</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -729,7 +726,7 @@
           <t>value_score</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
@@ -740,8 +737,8 @@
           <t>comps_percentile</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
-        <v>0.889</v>
+      <c r="B14" s="9" t="n">
+        <v>0.833</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -749,52 +746,67 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>dcf_margin</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Normalized (intrinsic − market) / market, clipped ±50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Honest caveats (read before acting)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
-        </is>
-      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
+          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
+          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
+          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
+          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>This is a SIGNAL screen, not an investment thesis. Verify with primary filings before acting.</t>
         </is>
@@ -804,6 +816,7 @@
   <mergeCells count="11">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
@@ -812,7 +825,6 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -878,8 +890,8 @@
           <t>Risk-free rate (10y Treasury)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
-        <v>0.04736999988555908</v>
+      <c r="B5" s="10" t="n">
+        <v>0.04690000057220459</v>
       </c>
     </row>
     <row r="6">
@@ -888,7 +900,7 @@
           <t>Equity risk premium (ERP)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -898,7 +910,7 @@
           <t>Beta (levered)</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -908,7 +920,7 @@
           <t>Credit spread over risk-free</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -918,7 +930,7 @@
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>0.21</v>
       </c>
     </row>
@@ -928,7 +940,7 @@
           <t>Equity weight (cap structure)</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="12" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -938,7 +950,7 @@
           <t>FCF growth (flat, faded avg)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>0.0725</v>
       </c>
     </row>
@@ -948,7 +960,7 @@
           <t>Terminal growth rate</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -958,7 +970,7 @@
           <t>Latest FCF ($, base year)</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <v>951000000</v>
       </c>
     </row>
@@ -968,7 +980,7 @@
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="14">
         <f>B5+B7*B6</f>
         <v/>
       </c>
@@ -979,18 +991,18 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="14">
         <f>(B5+B8)*(1-B9)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <f>B10*B15+(1-B10)*B16</f>
         <v/>
       </c>
@@ -1037,23 +1049,23 @@
           <t>Projected FCF</t>
         </is>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="17">
         <f>$B$13*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="17">
         <f>B22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="17">
         <f>C22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="17">
         <f>D22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="17">
         <f>E22*(1+$B$11)</f>
         <v/>
       </c>
@@ -1064,23 +1076,23 @@
           <t>Discount factor</t>
         </is>
       </c>
-      <c r="B23" s="17">
+      <c r="B23" s="18">
         <f>1/(1+$B$17)^1</f>
         <v/>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="18">
         <f>1/(1+$B$17)^2</f>
         <v/>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="18">
         <f>1/(1+$B$17)^3</f>
         <v/>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="18">
         <f>1/(1+$B$17)^4</f>
         <v/>
       </c>
-      <c r="F23" s="17">
+      <c r="F23" s="18">
         <f>1/(1+$B$17)^5</f>
         <v/>
       </c>
@@ -1091,23 +1103,23 @@
           <t>PV of FCF</t>
         </is>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="17">
         <f>B22*B23</f>
         <v/>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="17">
         <f>C22*C23</f>
         <v/>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="17">
         <f>D22*D23</f>
         <v/>
       </c>
-      <c r="E24" s="16">
+      <c r="E24" s="17">
         <f>E22*E23</f>
         <v/>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="17">
         <f>F22*F23</f>
         <v/>
       </c>
@@ -1118,7 +1130,7 @@
           <t>Sum of PV (explicit 5y)</t>
         </is>
       </c>
-      <c r="B26" s="16">
+      <c r="B26" s="17">
         <f>SUM(B24:F24)</f>
         <v/>
       </c>
@@ -1129,7 +1141,7 @@
           <t>Terminal value (Gordon)</t>
         </is>
       </c>
-      <c r="B27" s="16">
+      <c r="B27" s="17">
         <f>F22*(1+B12)/(B17-B12)</f>
         <v/>
       </c>
@@ -1140,18 +1152,18 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="B28" s="16">
+      <c r="B28" s="17">
         <f>B27/(1+B17)^5</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B29" s="19">
+      <c r="B29" s="20">
         <f>B26+B28</f>
         <v/>
       </c>
@@ -1176,7 +1188,7 @@
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="B32" s="12" t="n">
+      <c r="B32" s="13" t="n">
         <v>4160000000</v>
       </c>
     </row>
@@ -1186,7 +1198,7 @@
           <t>Plus: cash &amp; ST investments</t>
         </is>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B33" s="13" t="n">
         <v>540000000</v>
       </c>
     </row>
@@ -1196,7 +1208,7 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="B34" s="16">
+      <c r="B34" s="17">
         <f>B29-B32+B33</f>
         <v/>
       </c>
@@ -1207,17 +1219,17 @@
           <t>Diluted shares outstanding</t>
         </is>
       </c>
-      <c r="B35" s="20" t="n">
-        <v>120284976.9819495</v>
+      <c r="B35" s="21" t="n">
+        <v>120284979.3721973</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>Intrinsic per share</t>
         </is>
       </c>
-      <c r="B36" s="21">
+      <c r="B36" s="22">
         <f>B34/B35</f>
         <v/>
       </c>
@@ -1228,17 +1240,17 @@
           <t>Current market price</t>
         </is>
       </c>
-      <c r="B37" s="22" t="n">
-        <v>69.25</v>
+      <c r="B37" s="23" t="n">
+        <v>71.36</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B38" s="23">
+      <c r="B38" s="24">
         <f>(B36-B37)/B37</f>
         <v/>
       </c>
@@ -1258,158 +1270,158 @@
       <c r="H41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="inlineStr">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>WACC ↓ / TermG →</t>
         </is>
       </c>
-      <c r="B42" s="25">
+      <c r="B42" s="26">
         <f>$B$12+-0.01</f>
         <v/>
       </c>
-      <c r="C42" s="25">
+      <c r="C42" s="26">
         <f>$B$12+-0.005</f>
         <v/>
       </c>
-      <c r="D42" s="25">
+      <c r="D42" s="26">
         <f>$B$12+0.0</f>
         <v/>
       </c>
-      <c r="E42" s="25">
+      <c r="E42" s="26">
         <f>$B$12+0.005</f>
         <v/>
       </c>
-      <c r="F42" s="25">
+      <c r="F42" s="26">
         <f>$B$12+0.01</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="25">
+      <c r="A43" s="26">
         <f>$B$17+-0.01</f>
         <v/>
       </c>
-      <c r="B43" s="26">
+      <c r="B43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A43-B$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C43" s="26">
+      <c r="C43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A43-C$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D43" s="26">
+      <c r="D43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A43-D$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E43" s="26">
+      <c r="E43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A43-E$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F43" s="26">
+      <c r="F43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A43-F$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="25">
+      <c r="A44" s="26">
         <f>$B$17+-0.005</f>
         <v/>
       </c>
-      <c r="B44" s="26">
+      <c r="B44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A44-B$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C44" s="26">
+      <c r="C44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A44-C$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D44" s="26">
+      <c r="D44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A44-D$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E44" s="26">
+      <c r="E44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A44-E$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F44" s="26">
+      <c r="F44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A44-F$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="25">
+      <c r="A45" s="26">
         <f>$B$17+0.0</f>
         <v/>
       </c>
-      <c r="B45" s="26">
+      <c r="B45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A45-B$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C45" s="26">
+      <c r="C45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A45-C$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D45" s="27">
+      <c r="D45" s="28">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A45-D$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E45" s="26">
+      <c r="E45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A45-E$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F45" s="26">
+      <c r="F45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A45-F$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="25">
+      <c r="A46" s="26">
         <f>$B$17+0.005</f>
         <v/>
       </c>
-      <c r="B46" s="26">
+      <c r="B46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A46-B$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C46" s="26">
+      <c r="C46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A46-C$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D46" s="26">
+      <c r="D46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A46-D$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E46" s="26">
+      <c r="E46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A46-E$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F46" s="26">
+      <c r="F46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A46-F$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="25">
+      <c r="A47" s="26">
         <f>$B$17+0.01</f>
         <v/>
       </c>
-      <c r="B47" s="26">
+      <c r="B47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A47-B$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C47" s="26">
+      <c r="C47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A47-C$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D47" s="26">
+      <c r="D47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A47-D$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E47" s="26">
+      <c r="E47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A47-E$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F47" s="26">
+      <c r="F47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A47-F$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
@@ -1465,59 +1477,59 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C4" s="28" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="D4" s="28" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>P/E (TTM)</t>
         </is>
       </c>
-      <c r="E4" s="28" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="F4" s="28" t="inlineStr">
+      <c r="F4" s="29" t="inlineStr">
         <is>
           <t>EV/Revenue</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>BAH</t>
         </is>
       </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>Booz Allen Hamilton Holding Cor</t>
         </is>
       </c>
-      <c r="C5" s="30" t="n">
-        <v>8329734656</v>
-      </c>
-      <c r="D5" s="31" t="n">
-        <v>10.87</v>
-      </c>
-      <c r="E5" s="31" t="n">
-        <v>9.43</v>
-      </c>
-      <c r="F5" s="31" t="n">
-        <v>1.07</v>
+      <c r="C5" s="31" t="n">
+        <v>8583536128</v>
+      </c>
+      <c r="D5" s="32" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>1.08</v>
       </c>
     </row>
     <row r="6">
@@ -1531,17 +1543,17 @@
           <t>Aramark</t>
         </is>
       </c>
-      <c r="C6" s="32" t="n">
-        <v>15031741440</v>
-      </c>
-      <c r="D6" s="33" t="n">
-        <v>42.660446</v>
-      </c>
-      <c r="E6" s="33" t="n">
-        <v>14.996</v>
-      </c>
-      <c r="F6" s="33" t="n">
-        <v>1.085</v>
+      <c r="C6" s="33" t="n">
+        <v>14912096256</v>
+      </c>
+      <c r="D6" s="34" t="n">
+        <v>42.320892</v>
+      </c>
+      <c r="E6" s="34" t="n">
+        <v>14.944</v>
+      </c>
+      <c r="F6" s="34" t="n">
+        <v>1.081</v>
       </c>
     </row>
     <row r="7">
@@ -1555,15 +1567,15 @@
           <t>Grupo Aeroportuario del Sureste</t>
         </is>
       </c>
-      <c r="C7" s="32" t="n"/>
-      <c r="D7" s="33" t="n">
-        <v>14.910694</v>
-      </c>
-      <c r="E7" s="33" t="n">
-        <v>1.937</v>
-      </c>
-      <c r="F7" s="33" t="n">
-        <v>1</v>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="34" t="n">
+        <v>14.807384</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>1.935</v>
+      </c>
+      <c r="F7" s="34" t="n">
+        <v>0.999</v>
       </c>
     </row>
     <row r="8">
@@ -1577,17 +1589,17 @@
           <t>Acuity Inc.</t>
         </is>
       </c>
-      <c r="C8" s="32" t="n">
-        <v>9940698112</v>
-      </c>
-      <c r="D8" s="33" t="n">
-        <v>22.03517</v>
-      </c>
-      <c r="E8" s="33" t="n">
-        <v>13.995</v>
-      </c>
-      <c r="F8" s="33" t="n">
-        <v>2.266</v>
+      <c r="C8" s="33" t="n">
+        <v>10041580544</v>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>22.258793</v>
+      </c>
+      <c r="E8" s="34" t="n">
+        <v>13.617</v>
+      </c>
+      <c r="F8" s="34" t="n">
+        <v>2.205</v>
       </c>
     </row>
     <row r="9">
@@ -1601,17 +1613,17 @@
           <t>Clean Harbors, Inc.</t>
         </is>
       </c>
-      <c r="C9" s="32" t="n">
-        <v>16626399232</v>
-      </c>
-      <c r="D9" s="33" t="n">
-        <v>38.17818</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <v>16.126</v>
-      </c>
-      <c r="F9" s="33" t="n">
-        <v>3.086</v>
+      <c r="C9" s="33" t="n">
+        <v>16495222784</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>37.831112</v>
+      </c>
+      <c r="E9" s="34" t="n">
+        <v>16.084</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>3.083</v>
       </c>
     </row>
     <row r="10">
@@ -1625,14 +1637,14 @@
           <t>Crane Company</t>
         </is>
       </c>
-      <c r="C10" s="32" t="n"/>
-      <c r="D10" s="33" t="n">
-        <v>37.66899</v>
-      </c>
-      <c r="E10" s="33" t="n">
-        <v>24.719</v>
-      </c>
-      <c r="F10" s="33" t="n">
+      <c r="C10" s="33" t="n"/>
+      <c r="D10" s="34" t="n">
+        <v>38.117134</v>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>17.549</v>
+      </c>
+      <c r="F10" s="34" t="n">
         <v>5.058</v>
       </c>
     </row>
@@ -1647,17 +1659,17 @@
           <t>Mueller Industries, Inc.</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n">
-        <v>14857861120</v>
-      </c>
-      <c r="D11" s="33" t="n">
-        <v>17.49349</v>
-      </c>
-      <c r="E11" s="33" t="n">
-        <v>12.322</v>
-      </c>
-      <c r="F11" s="33" t="n">
-        <v>2.88</v>
+      <c r="C11" s="33" t="n">
+        <v>14617877504</v>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>17.210938</v>
+      </c>
+      <c r="E11" s="34" t="n">
+        <v>12.23</v>
+      </c>
+      <c r="F11" s="34" t="n">
+        <v>2.858</v>
       </c>
     </row>
     <row r="12">
@@ -1671,14 +1683,14 @@
           <t>Owens Corning Inc</t>
         </is>
       </c>
-      <c r="C12" s="32" t="n">
-        <v>11164849152</v>
-      </c>
-      <c r="D12" s="33" t="n"/>
-      <c r="E12" s="33" t="n">
-        <v>8.339</v>
-      </c>
-      <c r="F12" s="33" t="n">
+      <c r="C12" s="33" t="n">
+        <v>11518770176</v>
+      </c>
+      <c r="D12" s="34" t="n"/>
+      <c r="E12" s="34" t="n">
+        <v>8.342000000000001</v>
+      </c>
+      <c r="F12" s="34" t="n">
         <v>1.725</v>
       </c>
     </row>
@@ -1693,17 +1705,17 @@
           <t>Grupo Aeroportuario Del Pacific</t>
         </is>
       </c>
-      <c r="C13" s="32" t="n">
-        <v>12923200512</v>
-      </c>
-      <c r="D13" s="33" t="n">
-        <v>20.528357</v>
-      </c>
-      <c r="E13" s="33" t="n">
-        <v>86.309</v>
-      </c>
-      <c r="F13" s="33" t="n">
-        <v>58.389</v>
+      <c r="C13" s="33" t="n">
+        <v>12824129536</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>20.409563</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>85.45399999999999</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>57.81</v>
       </c>
     </row>
     <row r="15">
@@ -1712,15 +1724,15 @@
           <t>Peer median</t>
         </is>
       </c>
-      <c r="D15" s="34">
+      <c r="D15" s="35">
         <f>MEDIAN(D6:D13)</f>
         <v/>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="35">
         <f>MEDIAN(E6:E13)</f>
         <v/>
       </c>
-      <c r="F15" s="34">
+      <c r="F15" s="35">
         <f>MEDIAN(F6:F13)</f>
         <v/>
       </c>
@@ -1731,15 +1743,15 @@
           <t>Peer mean</t>
         </is>
       </c>
-      <c r="D16" s="34">
+      <c r="D16" s="35">
         <f>AVERAGE(D6:D13)</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="35">
         <f>AVERAGE(E6:E13)</f>
         <v/>
       </c>
-      <c r="F16" s="34">
+      <c r="F16" s="35">
         <f>AVERAGE(F6:F13)</f>
         <v/>
       </c>
@@ -1750,14 +1762,14 @@
           <t>Target percentile vs peers</t>
         </is>
       </c>
-      <c r="D17" s="35" t="n">
+      <c r="D17" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="35" t="n">
+      <c r="E17" s="36" t="n">
         <v>0.167</v>
       </c>
-      <c r="F17" s="35" t="n">
-        <v>0.167</v>
+      <c r="F17" s="36" t="n">
+        <v>0.333</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-07T17:44:53Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-04 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-07 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>180.78</v>
+        <v>179.82</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>72.81999999999999</v>
+        <v>75.86</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.483</v>
+        <v>1.37</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.0463100004196167</v>
+        <v>0.04654000282287598</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284971.3814886</v>
+        <v>120284971.2628526</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>72.81999999999999</v>
+        <v>75.86</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>8759151616</v>
+        <v>9124817920</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.43</v>
+        <v>11.91</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.699999999999999</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.1</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>14843728896</v>
+        <v>14789823488</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>42.126865</v>
+        <v>42.28947</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>14.901</v>
+        <v>14.82</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.078</v>
+        <v>1.072</v>
       </c>
     </row>
     <row r="7">
@@ -1569,13 +1569,13 @@
       </c>
       <c r="C7" s="33" t="n"/>
       <c r="D7" s="34" t="n">
-        <v>14.694355</v>
+        <v>14.694077</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>1.94</v>
+        <v>1.938</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.002</v>
+        <v>1.001</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>10372667392</v>
+        <v>10776199168</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>23.023256</v>
+        <v>23.887194</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>13.861</v>
+        <v>14.758</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>2.244</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16342404096</v>
+        <v>16268898304</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.708893</v>
+        <v>37.40261</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>16</v>
+        <v>15.853</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>3.067</v>
+        <v>3.039</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12941499392</v>
+        <v>12773301248</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>39.143356</v>
+        <v>38.567192</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>18.003</v>
+        <v>17.943</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>5.188</v>
+        <v>5.171</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>15139865600</v>
+        <v>15229445120</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>17.82552</v>
+        <v>17.93099</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>12.259</v>
+        <v>12.85</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>2.865</v>
+        <v>3.003</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>11649629184</v>
+        <v>12412224512</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>8.512</v>
+        <v>8.882999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.761</v>
+        <v>1.767</v>
       </c>
     </row>
     <row r="13">
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>13186198528</v>
+        <v>13292111872</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.985794</v>
+        <v>20.916666</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>85.75700000000001</v>
+        <v>87.279</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>58.015</v>
+        <v>59.045</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-08T17:40:08Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-07 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-08 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>179.82</v>
+        <v>179.57</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>75.86</v>
+        <v>76.05</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.37</v>
+        <v>1.361</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04654000282287598</v>
+        <v>0.04659999847412109</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284971.2628526</v>
+        <v>120284977.9881657</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>75.86</v>
+        <v>76.05</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9124817920</v>
+        <v>9147672576</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.91</v>
+        <v>11.94</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.970000000000001</v>
+        <v>10.17</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>14789823488</v>
+        <v>14712252416</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>42.28947</v>
+        <v>41.75373</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>14.82</v>
+        <v>14.753</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.072</v>
+        <v>1.067</v>
       </c>
     </row>
     <row r="7">
@@ -1569,13 +1569,13 @@
       </c>
       <c r="C7" s="33" t="n"/>
       <c r="D7" s="34" t="n">
-        <v>14.694077</v>
+        <v>14.623678</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>1.938</v>
+        <v>1.937</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>10776199168</v>
+        <v>10764223488</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>23.887194</v>
+        <v>23.86065</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>14.758</v>
+        <v>14.861</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>2.39</v>
+        <v>2.406</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16268898304</v>
+        <v>16267447296</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.40261</v>
+        <v>37.308716</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>15.853</v>
+        <v>15.876</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>3.039</v>
+        <v>3.043</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12773301248</v>
+        <v>12709142528</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>38.567192</v>
+        <v>38.30662</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>17.943</v>
+        <v>18.046</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>5.171</v>
+        <v>5.201</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>15229445120</v>
+        <v>15228338176</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>17.93099</v>
+        <v>17.929688</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>12.85</v>
+        <v>12.726</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>3.003</v>
+        <v>2.974</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>12412224512</v>
+        <v>12418547712</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>8.882999999999999</v>
+        <v>9.145</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.767</v>
+        <v>1.819</v>
       </c>
     </row>
     <row r="13">
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>13292111872</v>
+        <v>13251055616</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.916666</v>
+        <v>20.79365</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>87.279</v>
+        <v>87.505</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>59.045</v>
+        <v>59.198</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-10T17:42:54Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-09 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-10 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>179.57</v>
+        <v>177.93</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>76.05</v>
+        <v>77.26000000000001</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.361</v>
+        <v>1.303</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04659999847412109</v>
+        <v>0.04699999809265137</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284977.9881657</v>
+        <v>120284983.0701527</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>76.05</v>
+        <v>77.26000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9147672576</v>
+        <v>9293217792</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.94</v>
+        <v>12.13</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>10.17</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>14712252416</v>
+        <v>14599182336</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>41.75373</v>
+        <v>41.432835</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>14.753</v>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="C7" s="33" t="n"/>
       <c r="D7" s="34" t="n">
-        <v>14.623678</v>
+        <v>14.366279</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>1.937</v>
@@ -1590,10 +1590,10 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>10764223488</v>
+        <v>10663043072</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>23.86065</v>
+        <v>23.636364</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>14.861</v>
@@ -1614,10 +1614,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16267447296</v>
+        <v>16452993024</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.308716</v>
+        <v>37.73426</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>15.876</v>
@@ -1638,10 +1638,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12709142528</v>
+        <v>12737753088</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>38.30662</v>
+        <v>38.39286</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>18.046</v>
@@ -1662,10 +1662,10 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>15228338176</v>
+        <v>15321234432</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>17.929688</v>
+        <v>18.039062</v>
       </c>
       <c r="E11" s="34" t="n">
         <v>12.726</v>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>12418547712</v>
+        <v>12182192128</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
@@ -1708,10 +1708,10 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>13251055616</v>
+        <v>12864292864</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.79365</v>
+        <v>20.18674</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>87.505</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-08-11T17:42:55Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-10 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-11 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>177.93</v>
+        <v>178.58</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>77.26000000000001</v>
+        <v>78.015</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.303</v>
+        <v>1.289</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04699999809265137</v>
+        <v>0.04684000015258789</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284983.0701527</v>
+        <v>120284974.1203615</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>77.26000000000001</v>
+        <v>78.015</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9293217792</v>
+        <v>9384032256</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>12.13</v>
+        <v>12.25</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.17</v>
+        <v>10.35</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>14599182336</v>
+        <v>15961281536</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>41.432835</v>
+        <v>45.298508</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>14.753</v>
+        <v>14.708</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.067</v>
+        <v>1.064</v>
       </c>
     </row>
     <row r="7">
@@ -1569,13 +1569,13 @@
       </c>
       <c r="C7" s="33" t="n"/>
       <c r="D7" s="34" t="n">
-        <v>14.366279</v>
+        <v>14.449094</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>1.937</v>
+        <v>1.934</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1</v>
+        <v>0.998</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>10663043072</v>
+        <v>10748059648</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>23.636364</v>
+        <v>23.856478</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>14.861</v>
+        <v>14.614</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>2.406</v>
+        <v>2.366</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16452993024</v>
+        <v>16495486976</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.73426</v>
+        <v>37.877575</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>15.876</v>
+        <v>15.957</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>3.043</v>
+        <v>3.059</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12737753088</v>
+        <v>12760295424</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>38.39286</v>
+        <v>38.527924</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>18.046</v>
+        <v>18.005</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>5.201</v>
+        <v>5.189</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>15321234432</v>
+        <v>15283634176</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>18.039062</v>
+        <v>17.994791</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>12.726</v>
+        <v>12.736</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>2.974</v>
+        <v>2.977</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>12182192128</v>
+        <v>12482182144</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>9.145</v>
+        <v>9.012</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.819</v>
+        <v>1.793</v>
       </c>
     </row>
     <row r="13">
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>12864292864</v>
+        <v>12685193216</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.18674</v>
+        <v>20.09331</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>87.505</v>
+        <v>85.002</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>59.198</v>
+        <v>57.504</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-25T17:44:43Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-11 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-25 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>178.58</v>
+        <v>180.27</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>78.015</v>
+        <v>74.5399</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.289</v>
+        <v>1.418</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04684000015258789</v>
+        <v>0.0464300012588501</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284974.1203615</v>
+        <v>120284979.4002943</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>78.015</v>
+        <v>74.5399</v>
       </c>
     </row>
     <row r="38">
@@ -1516,20 +1516,20 @@
       </c>
       <c r="B5" s="30" t="inlineStr">
         <is>
-          <t>Booz Allen Hamilton Holding Cor</t>
+          <t>Booz Allen Hamilton Holding Corporation</t>
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9384032256</v>
+        <v>8966030336</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>12.25</v>
+        <v>11.7</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.35</v>
+        <v>10.09</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.17</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>15961281536</v>
+        <v>15622419456</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>45.298508</v>
+        <v>41.44056</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>14.708</v>
+        <v>14.99</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.064</v>
+        <v>1.091</v>
       </c>
     </row>
     <row r="7">
@@ -1569,13 +1569,13 @@
       </c>
       <c r="C7" s="33" t="n"/>
       <c r="D7" s="34" t="n">
-        <v>14.449094</v>
+        <v>13.636788</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>1.934</v>
+        <v>1.912</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>0.998</v>
+        <v>0.987</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>10748059648</v>
+        <v>10168057856</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>23.856478</v>
+        <v>22.569103</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>14.614</v>
+        <v>13.944</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>2.366</v>
+        <v>2.258</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16495486976</v>
+        <v>16485456896</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.877575</v>
+        <v>37.854546</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>15.957</v>
+        <v>16.122</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>3.059</v>
+        <v>3.09</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12760295424</v>
+        <v>11951379456</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>38.527924</v>
+        <v>36.02265</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>18.005</v>
+        <v>16.997</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>5.189</v>
+        <v>4.899</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>15283634176</v>
+        <v>13748635648</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>17.994791</v>
+        <v>16.1875</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>12.736</v>
+        <v>11.629</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>2.977</v>
+        <v>2.718</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>12482182144</v>
+        <v>11543083008</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>9.012</v>
+        <v>8.736000000000001</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.793</v>
+        <v>1.738</v>
       </c>
     </row>
     <row r="13">
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>12685193216</v>
+        <v>12427549696</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.09331</v>
+        <v>19.143906</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>85.002</v>
+        <v>80.877</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>57.504</v>
+        <v>54.714</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-29T17:42:55Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-25 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-29 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>180.27</v>
+        <v>177.12</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>74.5399</v>
+        <v>75.23999999999999</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.418</v>
+        <v>1.354</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.0464300012588501</v>
+        <v>0.0472</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284979.4002943</v>
+        <v>120284968.4210526</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>74.5399</v>
+        <v>75.23999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>8966030336</v>
+        <v>9050241024</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.7</v>
+        <v>11.81</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.09</v>
+        <v>10.1</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>1.14</v>
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>15622419456</v>
+        <v>15337704448</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>41.44056</v>
+        <v>40.685318</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>14.99</v>
+        <v>14.789</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.091</v>
+        <v>1.076</v>
       </c>
     </row>
     <row r="7">
@@ -1569,13 +1569,13 @@
       </c>
       <c r="C7" s="33" t="n"/>
       <c r="D7" s="34" t="n">
-        <v>13.636788</v>
+        <v>13.384615</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>1.912</v>
+        <v>1.908</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>0.987</v>
+        <v>0.985</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>10168057856</v>
+        <v>10033198080</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>22.569103</v>
+        <v>22.240213</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>13.944</v>
+        <v>13.887</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>2.258</v>
+        <v>2.249</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16485456896</v>
+        <v>16401525760</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.854546</v>
+        <v>37.75334</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>16.122</v>
+        <v>15.988</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>3.09</v>
+        <v>3.065</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>11951379456</v>
+        <v>11964674048</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>36.02265</v>
+        <v>36.125656</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>16.997</v>
+        <v>17.049</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.899</v>
+        <v>4.913</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13748635648</v>
+        <v>13890191360</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>16.1875</v>
+        <v>16.702127</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>11.629</v>
+        <v>11.777</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>2.718</v>
+        <v>2.753</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>11543083008</v>
+        <v>11314238464</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>8.736000000000001</v>
+        <v>8.582000000000001</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.738</v>
+        <v>1.707</v>
       </c>
     </row>
     <row r="13">
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>12427549696</v>
+        <v>12350197760</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>19.143906</v>
+        <v>19.059687</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>80.877</v>
+        <v>81.70099999999999</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>54.714</v>
+        <v>55.271</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-30T17:42:26Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-29 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.0472</v>
+        <v>0.04719999790191651</v>
       </c>
     </row>
     <row r="6">
@@ -1593,7 +1593,7 @@
         <v>10033198080</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>22.240213</v>
+        <v>22.67659</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>13.887</v>
@@ -1617,7 +1617,7 @@
         <v>16401525760</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.75334</v>
+        <v>37.616222</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>15.988</v>
@@ -1665,13 +1665,13 @@
         <v>13890191360</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>16.702127</v>
+        <v>16.354166</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>11.777</v>
+        <v>11.497</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>2.753</v>
+        <v>2.687</v>
       </c>
     </row>
     <row r="12">
@@ -1711,7 +1711,7 @@
         <v>12350197760</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>19.059687</v>
+        <v>19.730038</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>81.70099999999999</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-09-05T17:40:30Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>177.12</v>
+        <v>174.56</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>75.23999999999999</v>
+        <v>72.8</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.354</v>
+        <v>1.398</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04719999790191651</v>
+        <v>0.04783999919891357</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284968.4210526</v>
+        <v>120284975.8241758</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>75.23999999999999</v>
+        <v>72.8</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9050241024</v>
+        <v>8756746240</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.81</v>
+        <v>11.43</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.1</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.14</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>15337704448</v>
+        <v>14968629248</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>40.685318</v>
+        <v>39.985916</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>14.789</v>
+        <v>14.533</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.076</v>
+        <v>1.058</v>
       </c>
     </row>
     <row r="7">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="C7" s="33" t="n"/>
       <c r="D7" s="34" t="n">
-        <v>13.384615</v>
+        <v>13.402603</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>1.908</v>
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>10033198080</v>
+        <v>9999969280</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>22.67659</v>
+        <v>22.166555</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>13.887</v>
+        <v>13.843</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>2.249</v>
+        <v>2.242</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>16401525760</v>
+        <v>16738836480</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>37.616222</v>
+        <v>38.483013</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>15.988</v>
+        <v>16.27</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>3.065</v>
+        <v>3.119</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>11964674048</v>
+        <v>11831154688</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>36.125656</v>
+        <v>35.722515</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>17.049</v>
+        <v>16.87</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.913</v>
+        <v>4.862</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13890191360</v>
+        <v>14098102272</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>16.354166</v>
+        <v>16.385605</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>11.497</v>
+        <v>11.688</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>2.687</v>
+        <v>2.732</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>11314238464</v>
+        <v>10965633024</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>8.582000000000001</v>
+        <v>8.512</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.707</v>
+        <v>1.672</v>
       </c>
     </row>
     <row r="13">
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>12350197760</v>
+        <v>12386493440</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>19.730038</v>
+        <v>19.150873</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>81.70099999999999</v>
+        <v>81.935</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>55.271</v>
+        <v>55.429</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-09-06T17:40:02Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-06 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1547,7 @@
         <v>14968629248</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>39.985916</v>
+        <v>39.706295</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>14.533</v>
@@ -1665,7 +1665,7 @@
         <v>14098102272</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>16.385605</v>
+        <v>16.598959</v>
       </c>
       <c r="E11" s="34" t="n">
         <v>11.688</v>

</xml_diff>